<commit_message>
Rekap Mingguan: tambah tabel Akumulasi Per Periode 2-Mingguan
Di bawah tabel mingguan sekarang ada section 'AKUMULASI PER PERIODE
(2-MINGGUAN)' yang menggabungkan 2 minggu jadi 1 periode:
- Periode 1 = Minggu 1 + Minggu 2
- Periode 2 = Minggu 3 + Minggu 4
- Periode 3 = Minggu 5 (sendiri karena jumlah minggu ganjil)

Setiap periode punya semua kolom lengkap:
- Pagu Pangan (akumulasi 2 minggu) + Aktual + Selisih
- Pagu Operasional (akumulasi 2 minggu) + Aktual + Selisih
- Total Pagu + Total Aktual + Surplus/Defisit
- Status Periode: SURPLUS / DEFISIT / AMAN dengan warna otomatis
  (pakai conditional formatting sama seperti status mingguan)

Jadi user bisa langsung tau per 2 minggu itu surplus atau defisit,
tanpa perlu hitung manual.
</commit_message>
<xml_diff>
--- a/Template_Keuangan.xlsx
+++ b/Template_Keuangan.xlsx
@@ -3668,11 +3668,216 @@
         <f>SUM(K4:K8)</f>
       </c>
     </row>
+    <row r="11">
+</row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AKUMULASI PER PERIODE (2-MINGGUAN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Periode</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rentang Minggu</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pagu Pangan</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aktual Pangan</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Selisih Pangan</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pagu Operasional</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aktual Operasional</t>
+        </is>
+      </c>
+      <c r="H13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Selisih Operasional</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Pagu</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Aktual</t>
+        </is>
+      </c>
+      <c r="K13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surplus/Defisit</t>
+        </is>
+      </c>
+      <c r="L13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status Periode</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Periode 1</t>
+        </is>
+      </c>
+      <c r="B14" s="15">
+        <f>"Mg 1 - Mg 2"</f>
+      </c>
+      <c r="C14" s="7">
+        <f>SUM(C4:C5)</f>
+      </c>
+      <c r="D14" s="7">
+        <f>SUM(D4:D5)</f>
+      </c>
+      <c r="E14" s="17">
+        <f>C14-D14</f>
+      </c>
+      <c r="F14" s="7">
+        <f>SUM(F4:F5)</f>
+      </c>
+      <c r="G14" s="7">
+        <f>SUM(G4:G5)</f>
+      </c>
+      <c r="H14" s="17">
+        <f>F14-G14</f>
+      </c>
+      <c r="I14" s="7">
+        <f>C14+F14</f>
+      </c>
+      <c r="J14" s="7">
+        <f>D14+G14</f>
+      </c>
+      <c r="K14" s="17">
+        <f>I14-J14</f>
+      </c>
+      <c r="L14" s="29">
+        <f>IF(J14=0,"",IF(K14&gt;0,"SURPLUS",IF(K14&lt;0,"DEFISIT","AMAN")))</f>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Periode 2</t>
+        </is>
+      </c>
+      <c r="B15" s="15">
+        <f>"Mg 3 - Mg 4"</f>
+      </c>
+      <c r="C15" s="7">
+        <f>SUM(C6:C7)</f>
+      </c>
+      <c r="D15" s="7">
+        <f>SUM(D6:D7)</f>
+      </c>
+      <c r="E15" s="17">
+        <f>C15-D15</f>
+      </c>
+      <c r="F15" s="7">
+        <f>SUM(F6:F7)</f>
+      </c>
+      <c r="G15" s="7">
+        <f>SUM(G6:G7)</f>
+      </c>
+      <c r="H15" s="17">
+        <f>F15-G15</f>
+      </c>
+      <c r="I15" s="7">
+        <f>C15+F15</f>
+      </c>
+      <c r="J15" s="7">
+        <f>D15+G15</f>
+      </c>
+      <c r="K15" s="17">
+        <f>I15-J15</f>
+      </c>
+      <c r="L15" s="29">
+        <f>IF(J15=0,"",IF(K15&gt;0,"SURPLUS",IF(K15&lt;0,"DEFISIT","AMAN")))</f>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Periode 3</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>"Mg 5"</f>
+      </c>
+      <c r="C16" s="7">
+        <f>SUM(C8:C8)</f>
+      </c>
+      <c r="D16" s="7">
+        <f>SUM(D8:D8)</f>
+      </c>
+      <c r="E16" s="17">
+        <f>C16-D16</f>
+      </c>
+      <c r="F16" s="7">
+        <f>SUM(F8:F8)</f>
+      </c>
+      <c r="G16" s="7">
+        <f>SUM(G8:G8)</f>
+      </c>
+      <c r="H16" s="17">
+        <f>F16-G16</f>
+      </c>
+      <c r="I16" s="7">
+        <f>C16+F16</f>
+      </c>
+      <c r="J16" s="7">
+        <f>D16+G16</f>
+      </c>
+      <c r="K16" s="17">
+        <f>I16-J16</f>
+      </c>
+      <c r="L16" s="29">
+        <f>IF(J16=0,"",IF(K16&gt;0,"SURPLUS",IF(K16&lt;0,"DEFISIT","AMAN")))</f>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <conditionalFormatting sqref="L4:L8">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"SURPLUS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"DEFISIT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>"AMAN"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"BELUM"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L14:L16">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"SURPLUS"</formula>
     </cfRule>

</xml_diff>